<commit_message>
A23 follow-up checks; S1 Text analysis history; dictionary, SI and figure updates
</commit_message>
<xml_diff>
--- a/manuscript_v5/SI/S11_Table.xlsx
+++ b/manuscript_v5/SI/S11_Table.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A18_anchor_summary" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A18_anchor_counts" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A21_event_type" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A23_anchor_checks" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1210,6 +1211,532 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>anchor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>changed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>became_undetermined</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>became_determinate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>all determinate</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>carbo_cis_only</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>389</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>all determinate</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>389</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>all determinate</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>389</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>all determinate</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>389</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>added (117)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>carbo_cis_only</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>117</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>added (117)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>117</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>added (117)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>117</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>added (117)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>117</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>unflagged added (78)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>carbo_cis_only</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>78</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>unflagged added (78)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>78</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>unflagged added (78)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>78</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>unflagged added (78)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>78</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>discordant (4)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>carbo_cis_only</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>discordant (4)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>discordant (4)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>discordant (4)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>unflagged added resistant with RNA-seq</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>carbo_cis_only</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>unflagged added resistant with RNA-seq</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>unflagged added resistant with RNA-seq</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>unflagged added resistant with RNA-seq</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -33961,7 +34488,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>clean_resistant (recorded new tumour event, no flag); clean_sensitive (interval &gt;= 183 days, no flag); flagged (any flag, or a resistant call from a death counted as progression); negative_interval.</t>
+          <t>'clean' means that no specified provenance flag applied, not that the call is clinically verified. clean_resistant (recorded new tumour event, of any recorded or unrecorded type, no flag; 2 of the 12 added clean_resistant calls have an unrecorded event type); clean_sensitive (interval &gt;= 183 days, no flag); flagged (any flag, or a resistant call from a death counted as progression); negative_interval.</t>
         </is>
       </c>
     </row>

</xml_diff>